<commit_message>
Update project validation notes and user service dependencies
</commit_message>
<xml_diff>
--- a/LearningPath/Project-03-Persistent-User-Data/notes/validate_1_thru_3.xlsx
+++ b/LearningPath/Project-03-Persistent-User-Data/notes/validate_1_thru_3.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biome\Documents\PrimeServicesGroupKC\car-rental-microservices\LearningPath\Project-03-Persistent-User-Data\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3458141C-C74E-4885-8002-6A3ADBB37E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6577959A-AA07-40A1-BDC5-12DF8F88F578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6570" yWindow="1110" windowWidth="21510" windowHeight="11295" activeTab="1" xr2:uid="{88999B5D-CDC6-4AE0-A3D3-1B4E7E6906A7}"/>
+    <workbookView xWindow="6105" yWindow="3435" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{88999B5D-CDC6-4AE0-A3D3-1B4E7E6906A7}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="project_list" sheetId="1" r:id="rId1"/>
+    <sheet name="test_steps" sheetId="2" r:id="rId2"/>
+    <sheet name="git" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="196">
   <si>
     <t>Project</t>
   </si>
@@ -204,9 +205,6 @@
     <t>Project 1 — foundation checks</t>
   </si>
   <si>
-    <t>First verify Python and the project imports:</t>
-  </si>
-  <si>
     <t>python --version</t>
   </si>
   <si>
@@ -517,6 +515,120 @@
   </si>
   <si>
     <t>ORDER BY id;</t>
+  </si>
+  <si>
+    <t>Then:</t>
+  </si>
+  <si>
+    <t>SELECT * FROM alembic_version;</t>
+  </si>
+  <si>
+    <t>\q</t>
+  </si>
+  <si>
+    <t>Make sure secrets were NOT staged</t>
+  </si>
+  <si>
+    <t>git status --short</t>
+  </si>
+  <si>
+    <t>git ls-files | grep -E '(^|/)\.env$|(^|/)\.venv/'</t>
+  </si>
+  <si>
+    <t>Review the staged changes</t>
+  </si>
+  <si>
+    <t>git diff --cached --stat</t>
+  </si>
+  <si>
+    <t>git diff --cached</t>
+  </si>
+  <si>
+    <t>Space    → next page</t>
+  </si>
+  <si>
+    <t>b        → previous page</t>
+  </si>
+  <si>
+    <t>q        → quit</t>
+  </si>
+  <si>
+    <t>One important Alembic check</t>
+  </si>
+  <si>
+    <t>Make sure your migration is staged:</t>
+  </si>
+  <si>
+    <t>git status --short alembic/versions</t>
+  </si>
+  <si>
+    <t>git commit -m "Complete Project 3 persistent user data with PostgreSQL"</t>
+  </si>
+  <si>
+    <t>Then commit Project 3</t>
+  </si>
+  <si>
+    <t>git push</t>
+  </si>
+  <si>
+    <t>Verify Python and the project imports:</t>
+  </si>
+  <si>
+    <t>Verify git branch</t>
+  </si>
+  <si>
+    <t>git branch --show-current</t>
+  </si>
+  <si>
+    <t>Move into user-services</t>
+  </si>
+  <si>
+    <t>cd Webapp/services/user-service</t>
+  </si>
+  <si>
+    <t>Activate virtual environment</t>
+  </si>
+  <si>
+    <t>python -m pip check</t>
+  </si>
+  <si>
+    <t>Check installed dependencies</t>
+  </si>
+  <si>
+    <t>python -m pip show fastapi uvicorn sqlalchemy alembic psycopg pydantic pwdlib PyJWT pytest httpx</t>
+  </si>
+  <si>
+    <t>Check the important libraries</t>
+  </si>
+  <si>
+    <t>git remote -v</t>
+  </si>
+  <si>
+    <t>git branch -vv</t>
+  </si>
+  <si>
+    <t>git log --oneline -8</t>
+  </si>
+  <si>
+    <t>git ls-files Webapp/services/user-service/.env.example</t>
+  </si>
+  <si>
+    <t>git ls-files Webapp/services/user-service/.env</t>
+  </si>
+  <si>
+    <t>Move to root</t>
+  </si>
+  <si>
+    <t>python -c 'from app.main import app; print("Application import: PASS"); print("Title:", app.title)'</t>
+  </si>
+  <si>
+    <t>Verify the application can be imported - from user-service</t>
+  </si>
+  <si>
+    <t>python -m compileall -q app scripts tests</t>
+  </si>
+  <si>
+    <t>Check Python syntax</t>
   </si>
 </sst>
 </file>
@@ -540,12 +652,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -560,7 +678,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -571,6 +689,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1206,7 +1325,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A87B2EF9-2049-48A5-A4E0-2735FC487300}">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C167"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1216,682 +1335,907 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>54</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>55</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C4" t="s">
-        <v>56</v>
+      <c r="B4" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>57</v>
+        <v>178</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>58</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C11" t="s">
+    <row r="17" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C12" t="s">
+    <row r="18" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C13" t="s">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C16" t="s">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C17" t="s">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C18" t="s">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C35" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C37" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C41" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C44" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C22" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C46" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C48" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C50" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C24" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C26" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C52" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C28" t="s">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
         <v>77</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C30" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C32" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C33" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C34" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B35" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C36" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B37" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C38" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B39" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C40" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B41" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C42" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B43" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B44" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C45" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C46" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C47" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B48" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C49" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B50" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C51" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B52" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C53" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C54" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C55" t="s">
-        <v>104</v>
+      <c r="B55" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C56" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C57" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C58" t="s">
-        <v>107</v>
+        <v>82</v>
       </c>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C59" t="s">
-        <v>108</v>
+      <c r="B59" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C60" t="s">
-        <v>109</v>
+        <v>84</v>
       </c>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C61" t="s">
-        <v>110</v>
+      <c r="B61" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B62" t="s">
-        <v>111</v>
+      <c r="C62" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C63" t="s">
-        <v>100</v>
+      <c r="B63" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="64" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B64" t="s">
-        <v>112</v>
+      <c r="C64" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C65" t="s">
-        <v>113</v>
+      <c r="B65" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B66" t="s">
-        <v>114</v>
+      <c r="C66" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C67" t="s">
-        <v>115</v>
+      <c r="B67" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C69" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C70" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
     </row>
     <row r="71" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C71" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
     </row>
     <row r="72" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C72" t="s">
-        <v>118</v>
+      <c r="B72" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C73" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C74" t="s">
-        <v>110</v>
+      <c r="B74" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="75" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B75" t="s">
-        <v>120</v>
+      <c r="C75" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
-        <v>124</v>
+        <v>100</v>
       </c>
     </row>
     <row r="77" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C77" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="78" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C78" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C79" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C80" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
     </row>
     <row r="81" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C81" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
     </row>
     <row r="82" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C82" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C83" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="84" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C84" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C85" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B86" t="s">
         <v>110</v>
-      </c>
-    </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B85" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C86" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="87" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C87" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="88" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C88" t="s">
-        <v>104</v>
+      <c r="B88" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="89" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C89" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
     </row>
     <row r="90" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C90" t="s">
-        <v>126</v>
+      <c r="B90" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="91" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C91" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
     </row>
     <row r="92" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C92" t="s">
-        <v>128</v>
+      <c r="B92" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="93" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C93" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="94" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B94" t="s">
-        <v>129</v>
+      <c r="C94" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="95" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C95" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="96" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C96" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
     </row>
     <row r="97" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C97" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
     </row>
     <row r="98" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C98" t="s">
-        <v>130</v>
+        <v>109</v>
       </c>
     </row>
     <row r="99" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C99" t="s">
-        <v>131</v>
+      <c r="B99" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="100" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C100" t="s">
-        <v>107</v>
+      <c r="B100" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="101" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C101" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="102" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C102" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
     </row>
     <row r="103" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B103" t="s">
-        <v>132</v>
+      <c r="C103" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="104" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C104" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
     </row>
     <row r="105" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C105" t="s">
-        <v>103</v>
+        <v>121</v>
       </c>
     </row>
     <row r="106" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C106" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
     </row>
     <row r="107" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C107" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
     </row>
     <row r="108" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C108" t="s">
-        <v>133</v>
+        <v>109</v>
       </c>
     </row>
     <row r="109" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C109" t="s">
-        <v>134</v>
+      <c r="B109" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="110" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C110" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="111" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C111" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
     </row>
     <row r="112" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B112" t="s">
-        <v>135</v>
+      <c r="C112" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="113" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B113" t="s">
-        <v>136</v>
+      <c r="C113" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="114" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C114" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
     </row>
     <row r="115" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B115" t="s">
-        <v>138</v>
+      <c r="C115" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="116" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B116" t="s">
-        <v>139</v>
+      <c r="C116" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="117" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B117" t="s">
-        <v>140</v>
+      <c r="C117" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="118" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C118" t="s">
-        <v>89</v>
+      <c r="B118" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="119" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B119" t="s">
-        <v>141</v>
+      <c r="C119" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="120" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C120" t="s">
-        <v>142</v>
+        <v>102</v>
       </c>
     </row>
     <row r="121" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B121" t="s">
-        <v>143</v>
+      <c r="C121" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="122" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C122" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
     </row>
     <row r="123" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B123" t="s">
-        <v>145</v>
+      <c r="C123" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="124" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C124" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
     </row>
     <row r="125" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B125" t="s">
-        <v>146</v>
+      <c r="C125" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="126" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C126" t="s">
-        <v>71</v>
+        <v>109</v>
       </c>
     </row>
     <row r="127" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B127" t="s">
-        <v>147</v>
+        <v>131</v>
       </c>
     </row>
     <row r="128" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C128" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
     </row>
     <row r="129" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C129" t="s">
-        <v>142</v>
+        <v>102</v>
       </c>
     </row>
     <row r="130" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B130" t="s">
-        <v>148</v>
+      <c r="C130" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="131" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C131" t="s">
-        <v>149</v>
+        <v>129</v>
       </c>
     </row>
     <row r="132" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C132" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
     </row>
     <row r="133" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C133" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
     </row>
     <row r="134" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C134" t="s">
-        <v>152</v>
+        <v>108</v>
       </c>
     </row>
     <row r="135" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C135" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
     </row>
     <row r="136" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C136" t="s">
-        <v>154</v>
+      <c r="B136" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="137" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C137" t="s">
-        <v>155</v>
+      <c r="B137" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="138" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C138" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="139" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B139" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="140" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B140" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="141" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B141" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="142" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C142" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="143" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B143" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="144" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C144" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="145" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B145" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="146" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C146" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="147" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B147" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="148" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C148" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="149" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B149" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="150" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C150" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="151" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B151" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="152" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C152" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="153" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C153" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="154" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B154" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="155" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C155" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="156" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C156" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="157" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C157" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="158" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C158" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="159" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C159" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="160" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C160" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="161" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C161" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="162" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C162" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="163" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C163" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="139" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C139" t="s">
+    <row r="164" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C164" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="140" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C140" t="s">
+    <row r="165" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B165" t="s">
         <v>158</v>
+      </c>
+    </row>
+    <row r="166" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C166" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="167" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C167" t="s">
+        <v>160</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A11EE2E5-66D0-478C-8290-5C300AFF1F2D}">
+  <dimension ref="B1:D15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>